<commit_message>
publish: sync from 正本 2026-08-14T17:04:58Z
</commit_message>
<xml_diff>
--- a/plugins/osi-finance/assets/templates/請求管理台帳_テンプレート.xlsx
+++ b/plugins/osi-finance/assets/templates/請求管理台帳_テンプレート.xlsx
@@ -472,9 +472,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -574,7 +572,6 @@
           <t>（適格請求書 登録番号 T+13桁）</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -587,7 +584,6 @@
           <t>（例 000-0000）</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -600,7 +596,6 @@
           <t>（本店所在地）</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -613,7 +608,6 @@
           <t>（銀行名）</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -626,7 +620,6 @@
           <t>（支店名・店番）</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -639,7 +632,6 @@
           <t>普通</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -652,7 +644,6 @@
           <t>（口座番号）</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -665,7 +656,6 @@
           <t>（口座名義）</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -729,7 +719,6 @@
           <t>お客様負担</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -979,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1063,6 +1052,11 @@
           <t>備考</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>送付日</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">

</xml_diff>